<commit_message>
📊 Horarios actualizados Línea 141 - 5030
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-04.xlsx
+++ b/data/horarios-141-2026-10-04.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:27:28</t>
+          <t>Última actualización: 10:21:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:27:28</t>
+          <t>10:21:28</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>10:24</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:27:28</t>
+          <t>10:21:28</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:27:28</t>
+          <t>10:21:28</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>10:34</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:27:28</t>
+          <t>10:21:28</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:27:28</t>
+          <t>10:21:28</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>77</v>
+        <v>24</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:27:28</t>
+          <t>10:21:28</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:27:28</t>
+          <t>10:21:28</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>94</v>
+        <v>34</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:27:28</t>
+          <t>10:21:28</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>11:01</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>102</v>
+        <v>40</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,23 +673,273 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:27:28</t>
+          <t>10:21:28</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>105</v>
+        <v>43</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>10:21:28</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>47</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>10:21:28</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:16</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>55</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>10:21:28</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>63</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10:21:28</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>74</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>10:21:28</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>80</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10:21:28</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>83</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10:21:28</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>93</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>10:21:28</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>94</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>10:21:28</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>103</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>10:21:28</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>114</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -706,7 +956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -719,14 +969,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:27:28</t>
+          <t>Última actualización: 10:21:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -760,23 +1010,48 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:27:28</t>
+          <t>10:21:28</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>105</v>
+        <v>74</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>10:21:28</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>83</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -793,7 +1068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -806,14 +1081,116 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:27:28</t>
+          <t>Última actualización: 10:21:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>10:21:28</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>10:21:28</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>22</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>10:21:28</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>62</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5031
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-04.xlsx
+++ b/data/horarios-141-2026-10-04.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:21:28</t>
+          <t>Última actualización: 14:42:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -940,6 +940,481 @@
         <v>114</v>
       </c>
       <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>13</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>19</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>22</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>33</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>42</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>15:31</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>49</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>53</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>59</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>62</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>15:50</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>68</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>72</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>73</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>82</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>16:12</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>90</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>92</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>102</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>112</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>113</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -956,7 +1431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -969,14 +1444,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:21:28</t>
+          <t>Última actualización: 14:42:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1052,6 +1527,81 @@
         <v>83</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>13</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>22</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>53</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1068,7 +1618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1081,14 +1631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:21:28</t>
+          <t>Última actualización: 14:42:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1191,6 +1741,106 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>41</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>81</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>14:42:21</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>108</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5032
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-04.xlsx
+++ b/data/horarios-141-2026-10-04.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:42:21</t>
+          <t>Última actualización: 17:28:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 57</t>
         </is>
       </c>
     </row>
@@ -1415,6 +1415,481 @@
         <v>113</v>
       </c>
       <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>7</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>9</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>17</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>27</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>36</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>47</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>56</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>57</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>66</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>68</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>76</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>86</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>92</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>96</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>108</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>109</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>116</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>117</v>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1431,7 +1906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1444,14 +1919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:42:21</t>
+          <t>Última actualización: 17:28:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1602,6 +2077,131 @@
         <v>53</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>17</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>27</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>47</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>92</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>117</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1618,7 +2218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1631,14 +2231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:42:21</t>
+          <t>Última actualización: 17:28:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1839,6 +2439,56 @@
         <v>108</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>77</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>17:28:19</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>107</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5033
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-04.xlsx
+++ b/data/horarios-141-2026-10-04.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:28:19</t>
+          <t>Última actualización: 20:25:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 57</t>
+          <t>Total filas: 70</t>
         </is>
       </c>
     </row>
@@ -1890,6 +1890,331 @@
         <v>117</v>
       </c>
       <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>10</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>14</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>26</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>31</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>40</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>41</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>69</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>70</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>71</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>80</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>93</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>22:06</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>101</v>
+      </c>
+      <c r="E75" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1906,7 +2231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1919,14 +2244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:28:19</t>
+          <t>Última actualización: 20:25:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2202,6 +2527,81 @@
         <v>117</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>14</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>41</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2218,7 +2618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2231,14 +2631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:28:19</t>
+          <t>Última actualización: 20:25:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2489,6 +2889,81 @@
         <v>107</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>15</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>69</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>22:08</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>103</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5034
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-04.xlsx
+++ b/data/horarios-141-2026-10-04.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:25:57</t>
+          <t>Última actualización: 23:10:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 70</t>
+          <t>Total filas: 74</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>10:21:28</t>
+          <t>23:10:54</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>00:39</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>89</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -503,16 +503,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:24</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -528,16 +528,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -553,16 +553,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:34</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -578,16 +578,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -603,16 +603,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10:51</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -628,16 +628,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -653,16 +653,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11:01</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -678,16 +678,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>11:01</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -703,16 +703,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -728,16 +728,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>11:16</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -753,16 +753,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>11:24</t>
+          <t>11:16</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -778,16 +778,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>11:24</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -803,16 +803,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>11:41</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -828,16 +828,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -853,16 +853,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>11:54</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -878,16 +878,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:54</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -903,16 +903,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -928,16 +928,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,21 +948,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>14:42:21</t>
+          <t>10:21:28</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>14:46</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>4</v>
+        <v>114</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -978,16 +978,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:46</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1028,16 +1028,16 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1053,16 +1053,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1078,16 +1078,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1103,16 +1103,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>15:31</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1128,16 +1128,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:31</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1153,16 +1153,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1178,16 +1178,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1203,16 +1203,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>15:50</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1228,16 +1228,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1253,16 +1253,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:54</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1278,16 +1278,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1303,16 +1303,16 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>16:12</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1328,16 +1328,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:12</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1353,16 +1353,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1378,16 +1378,16 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1403,16 +1403,16 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>17:28:19</t>
+          <t>14:42:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>3</v>
+        <v>113</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1453,16 +1453,16 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1478,16 +1478,16 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1503,16 +1503,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1528,16 +1528,16 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1553,16 +1553,16 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1578,16 +1578,16 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1603,16 +1603,16 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1628,16 +1628,16 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1653,16 +1653,16 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1678,16 +1678,16 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1703,16 +1703,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1728,16 +1728,16 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:44</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1753,16 +1753,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1778,16 +1778,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1803,16 +1803,16 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1828,16 +1828,16 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1853,16 +1853,16 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1878,16 +1878,16 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>20:25:57</t>
+          <t>17:28:19</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1</v>
+        <v>117</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1928,16 +1928,16 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:26</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1953,16 +1953,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1978,16 +1978,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2003,16 +2003,16 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2028,16 +2028,16 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2053,16 +2053,16 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2078,16 +2078,16 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2103,16 +2103,16 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>21:35</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2128,16 +2128,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:35</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2153,16 +2153,16 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2178,16 +2178,16 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>21:58</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2203,18 +2203,118 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>93</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>20:25:57</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
           <t>22:06</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D75" t="n">
+      <c r="D76" t="n">
         <v>101</v>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>23:10:54</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>23:28</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>18</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>23:10:54</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>30</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>23:10:54</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>23:42</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>32</v>
+      </c>
+      <c r="E79" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2231,7 +2331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2244,14 +2344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:25:57</t>
+          <t>Última actualización: 23:10:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2602,6 +2702,56 @@
         <v>41</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>23:10:54</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>23:28</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>18</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>23:10:54</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>30</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2631,7 +2781,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:25:57</t>
+          <t>Última actualización: 23:10:54</t>
         </is>
       </c>
     </row>

</xml_diff>